<commit_message>
scenario: prologue 1-1 row 11, the bent manga is under the bookshelf, not the bed (author via main worker)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/シナリオ集/シナリオブラッシュアップ/第1章プロローグ｜シナリオ執筆用.xlsx
+++ b/シナリオ集/シナリオブラッシュアップ/第1章プロローグ｜シナリオ執筆用.xlsx
@@ -5313,9 +5313,9 @@
       <c r="D11" s="16" t="n"/>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>散らかったベッドの下には、
-昨日折れ曲がった漫画が落ちていた。
-どうやら昨日読みながら眠ってしまったみたい。</t>
+          <t>散らかった本棚の下に、
+昨日読んでいた漫画が折れ曲がって落ちていた。
+どうやら出しっぱなしで寝てしまったみたい。</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">

</xml_diff>

<commit_message>
scenario: prologue 1-1 rows 11-12 label, the bookshelf instead of the bed (author via main worker)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/シナリオ集/シナリオブラッシュアップ/第1章プロローグ｜シナリオ執筆用.xlsx
+++ b/シナリオ集/シナリオブラッシュアップ/第1章プロローグ｜シナリオ執筆用.xlsx
@@ -5320,7 +5320,7 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>アルシェのベッド周り</t>
+          <t>アルシェの本棚周り</t>
         </is>
       </c>
       <c r="H11" s="16" t="n"/>
@@ -5348,7 +5348,7 @@
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>アルシェのベッド周り</t>
+          <t>アルシェの本棚周り</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">

</xml_diff>